<commit_message>
Fix the merged files: FFmpeg
</commit_message>
<xml_diff>
--- a/ExcelFiles/FFmpeg.xlsx
+++ b/ExcelFiles/FFmpeg.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/muyeedahmed/Desktop/Gitcode/LLMVerification/ExcelFiles/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{428A9146-6CC9-244A-A984-24C6DE53C92C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{151C7979-DC41-BC42-98C4-B09B7181564A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1360" yWindow="500" windowWidth="27440" windowHeight="17500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="41480" yWindow="-21100" windowWidth="38400" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Commits" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="506" uniqueCount="314">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="552" uniqueCount="316">
   <si>
     <t>Commit Date</t>
   </si>
@@ -1059,6 +1059,12 @@
   </si>
   <si>
     <t>Deleted Code</t>
+  </si>
+  <si>
+    <t>No Change/Empty</t>
+  </si>
+  <si>
+    <t>Output Incorrect Function</t>
   </si>
 </sst>
 </file>
@@ -1578,7 +1584,7 @@
         <v>212</v>
       </c>
       <c r="K3" t="s">
-        <v>212</v>
+        <v>315</v>
       </c>
       <c r="L3" t="s">
         <v>216</v>
@@ -1889,7 +1895,7 @@
         <v>212</v>
       </c>
       <c r="K10" t="s">
-        <v>212</v>
+        <v>315</v>
       </c>
       <c r="L10" t="s">
         <v>218</v>
@@ -2077,7 +2083,7 @@
         <v>212</v>
       </c>
       <c r="K14" t="s">
-        <v>214</v>
+        <v>313</v>
       </c>
       <c r="L14" t="s">
         <v>216</v>
@@ -2124,7 +2130,7 @@
         <v>214</v>
       </c>
       <c r="K15" t="s">
-        <v>212</v>
+        <v>315</v>
       </c>
       <c r="L15" t="s">
         <v>216</v>
@@ -2259,7 +2265,7 @@
         <v>246</v>
       </c>
       <c r="K18" t="s">
-        <v>212</v>
+        <v>310</v>
       </c>
       <c r="L18" t="s">
         <v>216</v>
@@ -2401,7 +2407,7 @@
         <v>212</v>
       </c>
       <c r="K21" t="s">
-        <v>310</v>
+        <v>315</v>
       </c>
       <c r="L21" t="s">
         <v>216</v>
@@ -2589,7 +2595,7 @@
         <v>212</v>
       </c>
       <c r="K25" t="s">
-        <v>212</v>
+        <v>315</v>
       </c>
       <c r="L25" t="s">
         <v>218</v>
@@ -2639,7 +2645,7 @@
         <v>212</v>
       </c>
       <c r="K26" t="s">
-        <v>212</v>
+        <v>315</v>
       </c>
       <c r="L26" t="s">
         <v>218</v>
@@ -2686,7 +2692,7 @@
         <v>213</v>
       </c>
       <c r="K27" t="s">
-        <v>310</v>
+        <v>315</v>
       </c>
       <c r="L27" t="s">
         <v>216</v>
@@ -2865,7 +2871,7 @@
         <v>214</v>
       </c>
       <c r="K31" t="s">
-        <v>212</v>
+        <v>315</v>
       </c>
       <c r="L31" t="s">
         <v>216</v>
@@ -2912,6 +2918,9 @@
       <c r="I32" t="s">
         <v>212</v>
       </c>
+      <c r="K32" t="s">
+        <v>315</v>
+      </c>
       <c r="L32" t="s">
         <v>291</v>
       </c>
@@ -2956,6 +2965,9 @@
       <c r="I33" t="s">
         <v>255</v>
       </c>
+      <c r="K33" t="s">
+        <v>255</v>
+      </c>
       <c r="L33" t="s">
         <v>256</v>
       </c>
@@ -3000,6 +3012,9 @@
       <c r="I34" t="s">
         <v>211</v>
       </c>
+      <c r="K34" t="s">
+        <v>315</v>
+      </c>
       <c r="L34" t="s">
         <v>216</v>
       </c>
@@ -3044,6 +3059,9 @@
       <c r="I35" t="s">
         <v>212</v>
       </c>
+      <c r="K35" t="s">
+        <v>310</v>
+      </c>
       <c r="L35" t="s">
         <v>219</v>
       </c>
@@ -3088,6 +3106,9 @@
       <c r="I36" t="s">
         <v>212</v>
       </c>
+      <c r="K36" t="s">
+        <v>212</v>
+      </c>
       <c r="L36" t="s">
         <v>218</v>
       </c>
@@ -3132,6 +3153,9 @@
       <c r="I37" t="s">
         <v>212</v>
       </c>
+      <c r="K37" t="s">
+        <v>212</v>
+      </c>
       <c r="L37" t="s">
         <v>219</v>
       </c>
@@ -3176,6 +3200,9 @@
       <c r="I38" t="s">
         <v>212</v>
       </c>
+      <c r="K38" t="s">
+        <v>212</v>
+      </c>
       <c r="L38" t="s">
         <v>256</v>
       </c>
@@ -3220,6 +3247,9 @@
       <c r="I39" t="s">
         <v>212</v>
       </c>
+      <c r="K39" t="s">
+        <v>212</v>
+      </c>
       <c r="L39" t="s">
         <v>219</v>
       </c>
@@ -3264,6 +3294,9 @@
       <c r="I40" t="s">
         <v>213</v>
       </c>
+      <c r="K40" t="s">
+        <v>212</v>
+      </c>
       <c r="L40" t="s">
         <v>219</v>
       </c>
@@ -3296,6 +3329,9 @@
       <c r="I41" t="s">
         <v>255</v>
       </c>
+      <c r="K41" t="s">
+        <v>214</v>
+      </c>
       <c r="L41" t="s">
         <v>218</v>
       </c>
@@ -3340,6 +3376,9 @@
       <c r="I42" t="s">
         <v>255</v>
       </c>
+      <c r="K42" t="s">
+        <v>310</v>
+      </c>
       <c r="L42" t="s">
         <v>216</v>
       </c>
@@ -3384,6 +3423,9 @@
       <c r="I43" t="s">
         <v>212</v>
       </c>
+      <c r="K43" t="s">
+        <v>315</v>
+      </c>
       <c r="L43" t="s">
         <v>216</v>
       </c>
@@ -3428,6 +3470,9 @@
       <c r="I44" t="s">
         <v>214</v>
       </c>
+      <c r="K44" t="s">
+        <v>212</v>
+      </c>
       <c r="L44" t="s">
         <v>216</v>
       </c>
@@ -3460,6 +3505,9 @@
       <c r="I45" t="s">
         <v>246</v>
       </c>
+      <c r="K45" t="s">
+        <v>212</v>
+      </c>
       <c r="L45" t="s">
         <v>216</v>
       </c>
@@ -3504,6 +3552,9 @@
       <c r="I46" t="s">
         <v>214</v>
       </c>
+      <c r="K46" t="s">
+        <v>310</v>
+      </c>
       <c r="L46" t="s">
         <v>216</v>
       </c>
@@ -3548,6 +3599,9 @@
       <c r="I47" t="s">
         <v>212</v>
       </c>
+      <c r="K47" t="s">
+        <v>315</v>
+      </c>
       <c r="L47" t="s">
         <v>216</v>
       </c>
@@ -3593,6 +3647,9 @@
       <c r="I48" t="s">
         <v>235</v>
       </c>
+      <c r="K48" t="s">
+        <v>315</v>
+      </c>
       <c r="L48" t="s">
         <v>219</v>
       </c>
@@ -3637,6 +3694,9 @@
       <c r="I49" t="s">
         <v>212</v>
       </c>
+      <c r="K49" t="s">
+        <v>315</v>
+      </c>
       <c r="L49" t="s">
         <v>220</v>
       </c>
@@ -3681,6 +3741,9 @@
       <c r="I50" t="s">
         <v>215</v>
       </c>
+      <c r="K50" t="s">
+        <v>310</v>
+      </c>
       <c r="L50" t="s">
         <v>216</v>
       </c>
@@ -3713,6 +3776,9 @@
       <c r="I51" t="s">
         <v>213</v>
       </c>
+      <c r="K51" t="s">
+        <v>315</v>
+      </c>
       <c r="L51" t="s">
         <v>216</v>
       </c>
@@ -3757,6 +3823,9 @@
       <c r="I52" t="s">
         <v>212</v>
       </c>
+      <c r="K52" t="s">
+        <v>212</v>
+      </c>
       <c r="L52" t="s">
         <v>217</v>
       </c>
@@ -3804,6 +3873,9 @@
       <c r="I53" t="s">
         <v>214</v>
       </c>
+      <c r="K53" t="s">
+        <v>212</v>
+      </c>
       <c r="L53" t="s">
         <v>219</v>
       </c>
@@ -3848,6 +3920,9 @@
       <c r="I54" t="s">
         <v>212</v>
       </c>
+      <c r="K54" t="s">
+        <v>310</v>
+      </c>
       <c r="L54" t="s">
         <v>256</v>
       </c>
@@ -3892,6 +3967,9 @@
       <c r="I55" t="s">
         <v>212</v>
       </c>
+      <c r="K55" t="s">
+        <v>315</v>
+      </c>
       <c r="L55" t="s">
         <v>218</v>
       </c>
@@ -3936,6 +4014,9 @@
       <c r="I56" t="s">
         <v>214</v>
       </c>
+      <c r="K56" t="s">
+        <v>213</v>
+      </c>
       <c r="L56" t="s">
         <v>216</v>
       </c>
@@ -3980,6 +4061,9 @@
       <c r="I57" t="s">
         <v>214</v>
       </c>
+      <c r="K57" t="s">
+        <v>214</v>
+      </c>
       <c r="L57" t="s">
         <v>216</v>
       </c>
@@ -4024,6 +4108,9 @@
       <c r="I58" t="s">
         <v>213</v>
       </c>
+      <c r="K58" t="s">
+        <v>213</v>
+      </c>
       <c r="L58" t="s">
         <v>220</v>
       </c>
@@ -4068,6 +4155,9 @@
       <c r="I59" t="s">
         <v>213</v>
       </c>
+      <c r="K59" t="s">
+        <v>213</v>
+      </c>
       <c r="L59" t="s">
         <v>216</v>
       </c>
@@ -4100,6 +4190,9 @@
       <c r="I60" t="s">
         <v>235</v>
       </c>
+      <c r="K60" t="s">
+        <v>315</v>
+      </c>
       <c r="L60" t="s">
         <v>216</v>
       </c>
@@ -4144,6 +4237,9 @@
       <c r="I61" t="s">
         <v>212</v>
       </c>
+      <c r="K61" t="s">
+        <v>315</v>
+      </c>
       <c r="L61" t="s">
         <v>216</v>
       </c>
@@ -4188,6 +4284,9 @@
       <c r="I62" t="s">
         <v>212</v>
       </c>
+      <c r="K62" t="s">
+        <v>310</v>
+      </c>
       <c r="L62" t="s">
         <v>216</v>
       </c>
@@ -4232,6 +4331,9 @@
       <c r="I63" t="s">
         <v>215</v>
       </c>
+      <c r="K63" t="s">
+        <v>315</v>
+      </c>
       <c r="L63" t="s">
         <v>216</v>
       </c>
@@ -4276,6 +4378,12 @@
       <c r="I64" t="s">
         <v>214</v>
       </c>
+      <c r="J64" t="s">
+        <v>314</v>
+      </c>
+      <c r="K64" t="s">
+        <v>310</v>
+      </c>
       <c r="L64" t="s">
         <v>216</v>
       </c>
@@ -4308,6 +4416,9 @@
       <c r="I65" t="s">
         <v>280</v>
       </c>
+      <c r="K65" t="s">
+        <v>315</v>
+      </c>
       <c r="L65" t="s">
         <v>216</v>
       </c>
@@ -4352,6 +4463,9 @@
       <c r="I66" t="s">
         <v>212</v>
       </c>
+      <c r="K66" t="s">
+        <v>315</v>
+      </c>
       <c r="L66" t="s">
         <v>216</v>
       </c>
@@ -4396,6 +4510,9 @@
       <c r="I67" t="s">
         <v>212</v>
       </c>
+      <c r="K67" t="s">
+        <v>212</v>
+      </c>
       <c r="L67" t="s">
         <v>218</v>
       </c>
@@ -4440,6 +4557,9 @@
       <c r="I68" t="s">
         <v>255</v>
       </c>
+      <c r="K68" t="s">
+        <v>315</v>
+      </c>
       <c r="L68" t="s">
         <v>218</v>
       </c>
@@ -4484,6 +4604,9 @@
       <c r="I69" t="s">
         <v>212</v>
       </c>
+      <c r="K69" t="s">
+        <v>212</v>
+      </c>
       <c r="L69" t="s">
         <v>220</v>
       </c>
@@ -4529,6 +4652,9 @@
       <c r="I70" t="s">
         <v>214</v>
       </c>
+      <c r="K70" t="s">
+        <v>214</v>
+      </c>
       <c r="L70" t="s">
         <v>291</v>
       </c>
@@ -4573,6 +4699,9 @@
       <c r="I71" t="s">
         <v>212</v>
       </c>
+      <c r="K71" t="s">
+        <v>315</v>
+      </c>
       <c r="L71" t="s">
         <v>219</v>
       </c>
@@ -4617,6 +4746,9 @@
       <c r="I72" t="s">
         <v>212</v>
       </c>
+      <c r="K72" t="s">
+        <v>315</v>
+      </c>
       <c r="L72" t="s">
         <v>219</v>
       </c>
@@ -4661,6 +4793,9 @@
       <c r="I73" t="s">
         <v>212</v>
       </c>
+      <c r="K73" t="s">
+        <v>315</v>
+      </c>
       <c r="L73" t="s">
         <v>220</v>
       </c>
@@ -4705,6 +4840,9 @@
       <c r="I74" t="s">
         <v>255</v>
       </c>
+      <c r="K74" t="s">
+        <v>315</v>
+      </c>
       <c r="L74" t="s">
         <v>218</v>
       </c>
@@ -4749,6 +4887,9 @@
       <c r="I75" t="s">
         <v>212</v>
       </c>
+      <c r="K75" t="s">
+        <v>213</v>
+      </c>
       <c r="L75" t="s">
         <v>216</v>
       </c>
@@ -4780,6 +4921,9 @@
       </c>
       <c r="I76" t="s">
         <v>255</v>
+      </c>
+      <c r="K76" t="s">
+        <v>212</v>
       </c>
       <c r="L76" t="s">
         <v>220</v>

</xml_diff>